<commit_message>
Update Doctor Schedule Admin TestCase
</commit_message>
<xml_diff>
--- a/TestCases/Doctor_Schedule_Admin_TestCase.xlsx
+++ b/TestCases/Doctor_Schedule_Admin_TestCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDC10E0-552A-4614-92B9-937311EEC9FA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8696F6DC-1BC0-4181-BEAB-1DE19EB0C63E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="155">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -413,6 +413,178 @@
   <si>
     <t>Sau khi thêm lịch thành công, form được reset đúng về các giá trị mặc định.</t>
   </si>
+  <si>
+    <t>7. Kiểm tra chức năng lọc và xem lịch làm việc</t>
+  </si>
+  <si>
+    <t>TC-DS-ADMIN-014</t>
+  </si>
+  <si>
+    <t>Kiểm tra Admin có thể lọc lịch làm việc theo một bác sĩ cụ thể.</t>
+  </si>
+  <si>
+    <t>1: Đăng nhập bằng tài khoản Admin.
+2: Mở trang Quản lý lịch làm việc.
+3: Tại mục Lọc lịch làm việc, chọn bác sĩ Tran Binh.
+4: Quan sát bảng Lịch làm việc theo tuần.
+5: Kiểm tra các lịch đang hiển thị trong tuần hiện tại.</t>
+  </si>
+  <si>
+    <t>Bảng Lịch làm việc theo tuần chỉ hiển thị lịch của bác sĩ Tran Binh; lịch của các bác sĩ khác không được hiển thị.</t>
+  </si>
+  <si>
+    <t>TCDsAdmin14</t>
+  </si>
+  <si>
+    <t>Bộ lọc theo bác sĩ hoạt động đúng; sau khi chọn Tran Binh, bảng lịch theo tuần chỉ hiển thị lịch của bác sĩ Tran Binh.</t>
+  </si>
+  <si>
+    <t>TC-DS-ADMIN-015</t>
+  </si>
+  <si>
+    <t>Kiểm tra hiển thị lại lịch của tất cả bác sĩ sau khi bỏ điều kiện lọc.</t>
+  </si>
+  <si>
+    <t>1: Tại mục Lọc lịch làm việc, chọn bác sĩ Tran Binh.
+2: Xác nhận bảng tuần chỉ hiển thị lịch của Tran Binh.
+3: Chọn lại Tất cả bác sĩ.
+4: Quan sát bảng Lịch làm việc theo tuần.</t>
+  </si>
+  <si>
+    <t>Hệ thống bỏ điều kiện lọc và hiển thị lại lịch làm việc của tất cả bác sĩ trong tuần đang xem.</t>
+  </si>
+  <si>
+    <t>TCDsAdmin15_1, TCDsAdmin15_2</t>
+  </si>
+  <si>
+    <t>Hệ thống khôi phục đúng dữ liệu khi bỏ điều kiện lọc theo bác sĩ; các lịch của Tran Binh, Pham Dung, Ly Minh và Vu Thinh được hiển thị lại trong bảng tuần.</t>
+  </si>
+  <si>
+    <t>TC-DS-ADMIN-016</t>
+  </si>
+  <si>
+    <t>Kiểm tra Admin có thể chuyển sang tuần trước để xem lịch làm việc.</t>
+  </si>
+  <si>
+    <t>1: Mở trang Quản lý lịch làm việc.
+2: Ghi nhận khoảng thời gian của tuần đang hiển thị.
+3: Nhấn nút Tuần trước.
+4: Quan sát khoảng thời gian tại mục Tuần làm việc.
+5: Quan sát ngày và dữ liệu trong bảng Lịch làm việc theo tuần.</t>
+  </si>
+  <si>
+    <t>Hệ thống chuyển về tuần liền trước; khoảng ngày và các cột ngày trong bảng tuần được cập nhật đúng theo tuần mới; dữ liệu lịch hiển thị tương ứng với tuần được chọn.</t>
+  </si>
+  <si>
+    <t>TCDsAdmin16_1, TCDsAdmin16_2</t>
+  </si>
+  <si>
+    <t>Chức năng chuyển về tuần trước hoạt động đúng; khoảng thời gian và dữ liệu lịch được hiển thị theo tuần đã chọn.</t>
+  </si>
+  <si>
+    <t>TC-DS-ADMIN-017</t>
+  </si>
+  <si>
+    <t>Kiểm tra Admin có thể chuyển sang tuần sau để xem lịch làm việc.</t>
+  </si>
+  <si>
+    <t>1: Mở trang Quản lý lịch làm việc.
+2: Ghi nhận khoảng thời gian của tuần đang hiển thị.
+3: Nhấn nút Tuần sau.
+4: Quan sát khoảng thời gian tại mục Tuần làm việc.
+5: Quan sát ngày và dữ liệu trong bảng Lịch làm việc theo tuần.</t>
+  </si>
+  <si>
+    <t>Hệ thống chuyển sang tuần liền sau; khoảng ngày và các cột ngày trong bảng tuần được cập nhật đúng theo tuần mới; dữ liệu lịch hiển thị tương ứng với tuần được chọn.</t>
+  </si>
+  <si>
+    <t>TCDsAdmin17_1, TCDsAdmin17_2</t>
+  </si>
+  <si>
+    <t>Chức năng chuyển sang tuần sau hoạt động đúng; khoảng thời gian và dữ liệu lịch được hiển thị theo tuần đã chọn.</t>
+  </si>
+  <si>
+    <t>8. Kiểm tra chức năng sửa lịch làm việc</t>
+  </si>
+  <si>
+    <t>TC-DS-ADMIN-018</t>
+  </si>
+  <si>
+    <t>Kiểm tra Admin cập nhật lịch làm việc của bác sĩ thành công.</t>
+  </si>
+  <si>
+    <t>1: Đăng nhập bằng tài khoản Admin.
+2: Mở trang Quản lý lịch làm việc.
+3: Tại Danh sách lịch làm việc, chọn một lịch đã tồn tại và nhấn Sửa.
+4: Kiểm tra thông tin lịch được hiển thị trên form Cập nhật lịch làm việc.
+5: Thay đổi Trạng thái từ Có lịch làm việc thành Không làm việc.
+6: Thay đổi Ghi chú thành Nghỉ.
+7: Nhấn Cập nhật.
+8: Kiểm tra thông báo của hệ thống.
+9: Kiểm tra lại lịch trong Danh sách lịch làm việc và bảng Lịch làm việc theo tuần.</t>
+  </si>
+  <si>
+    <t>Hệ thống cập nhật lịch thành công; trạng thái và ghi chú được thay đổi đúng, không tạo thêm bản ghi mới và thông tin được hiển thị đúng trong danh sách và bảng tuần.</t>
+  </si>
+  <si>
+    <t>TCDsAdmin18_1, TCDsAdmin18_2</t>
+  </si>
+  <si>
+    <t>Hệ thống phát sinh lỗi HTTP 400 khi cập nhật lịch làm việc và không lưu thông tin thay đổi.</t>
+  </si>
+  <si>
+    <t>TCDsAdminRetest18_1, TCDsAdminRetest18_2, TCDsAdminRetest18_3</t>
+  </si>
+  <si>
+    <t>TC-DS-ADMIN-019</t>
+  </si>
+  <si>
+    <t>Kiểm tra chức năng Hủy sửa không làm thay đổi dữ liệu lịch.</t>
+  </si>
+  <si>
+    <t>1: Chọn một lịch hiện có trong Danh sách lịch làm việc và ghi nhận thông tin ban đầu.
+2: Nhấn Sửa.
+3: Thay đổi một số giá trị trên form nhưng chưa nhấn Cập nhật.
+4: Nhấn Hủy sửa.
+5: Quan sát lại form.
+6: Kiểm tra lịch tương ứng trong Danh sách lịch làm việc.</t>
+  </si>
+  <si>
+    <t>Hệ thống thoát chế độ cập nhật và đưa form về trạng thái thêm lịch mặc định; các thay đổi chưa được lưu không làm thay đổi dữ liệu của lịch trong Danh sách lịch làm việc.</t>
+  </si>
+  <si>
+    <t>TCDsAdmin19_1, TCDsAdmin19_2, TCDsAdmin19_3</t>
+  </si>
+  <si>
+    <t>Chức năng Hủy sửa hoạt động đúng, không làm thay đổi dữ liệu của lịch hiện có.</t>
+  </si>
+  <si>
+    <t>9. Kiểm tra chức năng xóa lịch làm việc</t>
+  </si>
+  <si>
+    <t>TC-DS-ADMIN-020</t>
+  </si>
+  <si>
+    <t>Kiểm tra Admin có thể xóa một lịch làm việc đã tồn tại.</t>
+  </si>
+  <si>
+    <t>1: Tạo hoặc xác định một lịch dùng riêng cho kiểm thử xóa.
+2: Kiểm tra lịch đang tồn tại trong Danh sách lịch làm việc.
+3: Nhấn nút Xóa tại lịch đó.
+4: Xác nhận thao tác xóa nếu hệ thống yêu cầu xác nhận.
+5: Chờ hệ thống xử lý.
+6: Kiểm tra lại Danh sách lịch làm việc.
+7: Kiểm tra bảng Lịch làm việc theo tuần.</t>
+  </si>
+  <si>
+    <t>Hệ thống xóa lịch thành công; lịch đã xóa không còn xuất hiện trong Danh sách lịch làm việc và không còn hiển thị trong bảng Lịch làm việc theo tuần.</t>
+  </si>
+  <si>
+    <t>TCDsAdmin20_1, TCDsAdmin20_2, TCDsAdmin20_3</t>
+  </si>
+  <si>
+    <t>Chức năng xóa lịch hoạt động đúng; hệ thống yêu cầu xác nhận trước khi xóa và loại bỏ lịch khỏi danh sách sau khi xác nhận.</t>
+  </si>
 </sst>
 </file>
 
@@ -434,6 +606,10 @@
       <name val="Tahoma"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="MS PGothic"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -443,10 +619,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="MS PGothic"/>
     </font>
     <font>
       <b/>
@@ -651,12 +823,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -672,10 +844,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -691,17 +863,14 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -710,12 +879,12 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -731,13 +900,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -960,7 +1129,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1004"/>
+  <dimension ref="A1:AA1003"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -979,9 +1148,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1008,9 +1177,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1039,11 +1208,11 @@
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="28"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="27"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1072,11 +1241,11 @@
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="28"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="27"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1105,11 +1274,11 @@
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="26"/>
-      <c r="D5" s="28"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="27"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1139,7 +1308,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>6</v>
@@ -1176,13 +1345,13 @@
         <v>7</v>
       </c>
       <c r="B7" s="6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="8">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -1238,39 +1407,39 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="37" t="s">
+      <c r="D9" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="35" t="s">
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="38" t="s">
+      <c r="H9" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="38" t="s">
+      <c r="I9" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="38" t="s">
+      <c r="J9" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="38" t="s">
+      <c r="K9" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="38" t="s">
+      <c r="L9" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="38" t="s">
+      <c r="M9" s="37" t="s">
         <v>19</v>
       </c>
       <c r="N9" s="3"/>
@@ -1289,19 +1458,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="27"/>
-      <c r="L10" s="27"/>
-      <c r="M10" s="27"/>
+      <c r="A10" s="26"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1319,18 +1488,18 @@
     </row>
     <row r="11" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="25"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1347,21 +1516,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
-      <c r="M12" s="28"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="27"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1387,11 +1556,11 @@
       <c r="C13" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
       <c r="G13" s="17" t="s">
         <v>27</v>
       </c>
@@ -1423,21 +1592,21 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="40" t="s">
+      <c r="A14" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
-      <c r="M14" s="28"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="25"/>
+      <c r="M14" s="27"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1463,11 +1632,11 @@
       <c r="C15" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="D15" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
       <c r="G15" s="17" t="s">
         <v>34</v>
       </c>
@@ -1514,11 +1683,11 @@
       <c r="C16" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
       <c r="G16" s="17" t="s">
         <v>41</v>
       </c>
@@ -1565,11 +1734,11 @@
       <c r="C17" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
       <c r="G17" s="17" t="s">
         <v>47</v>
       </c>
@@ -1607,21 +1776,21 @@
       <c r="AA17" s="3"/>
     </row>
     <row r="18" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A18" s="40" t="s">
+      <c r="A18" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="28"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="25"/>
+      <c r="M18" s="27"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -1647,11 +1816,11 @@
       <c r="C19" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
       <c r="G19" s="17" t="s">
         <v>54</v>
       </c>
@@ -1692,11 +1861,11 @@
       <c r="C20" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
       <c r="G20" s="17" t="s">
         <v>60</v>
       </c>
@@ -1728,34 +1897,34 @@
       <c r="AA20" s="3"/>
     </row>
     <row r="21" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="42"/>
-      <c r="O21" s="32"/>
-      <c r="P21" s="32"/>
-      <c r="Q21" s="32"/>
-      <c r="R21" s="32"/>
-      <c r="S21" s="32"/>
-      <c r="T21" s="32"/>
-      <c r="U21" s="32"/>
-      <c r="V21" s="32"/>
-      <c r="W21" s="32"/>
-      <c r="X21" s="32"/>
-      <c r="Y21" s="32"/>
-      <c r="Z21" s="32"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="25"/>
+      <c r="L21" s="25"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="41"/>
+      <c r="O21" s="31"/>
+      <c r="P21" s="31"/>
+      <c r="Q21" s="31"/>
+      <c r="R21" s="31"/>
+      <c r="S21" s="31"/>
+      <c r="T21" s="31"/>
+      <c r="U21" s="31"/>
+      <c r="V21" s="31"/>
+      <c r="W21" s="31"/>
+      <c r="X21" s="31"/>
+      <c r="Y21" s="31"/>
+      <c r="Z21" s="31"/>
       <c r="AA21" s="3"/>
     </row>
     <row r="22" spans="1:27" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1768,12 +1937,12 @@
       <c r="C22" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="24" t="s">
+      <c r="E22" s="25"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="23" t="s">
         <v>67</v>
       </c>
       <c r="H22" s="18">
@@ -1804,34 +1973,34 @@
       <c r="AA22" s="3"/>
     </row>
     <row r="23" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26"/>
-      <c r="L23" s="26"/>
-      <c r="M23" s="28"/>
-      <c r="N23" s="43"/>
-      <c r="O23" s="32"/>
-      <c r="P23" s="32"/>
-      <c r="Q23" s="32"/>
-      <c r="R23" s="32"/>
-      <c r="S23" s="32"/>
-      <c r="T23" s="32"/>
-      <c r="U23" s="32"/>
-      <c r="V23" s="32"/>
-      <c r="W23" s="32"/>
-      <c r="X23" s="32"/>
-      <c r="Y23" s="32"/>
-      <c r="Z23" s="32"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="42"/>
+      <c r="O23" s="31"/>
+      <c r="P23" s="31"/>
+      <c r="Q23" s="31"/>
+      <c r="R23" s="31"/>
+      <c r="S23" s="31"/>
+      <c r="T23" s="31"/>
+      <c r="U23" s="31"/>
+      <c r="V23" s="31"/>
+      <c r="W23" s="31"/>
+      <c r="X23" s="31"/>
+      <c r="Y23" s="31"/>
+      <c r="Z23" s="31"/>
       <c r="AA23" s="3"/>
     </row>
     <row r="24" spans="1:27" ht="126" customHeight="1" x14ac:dyDescent="0.25">
@@ -1844,11 +2013,11 @@
       <c r="C24" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="41" t="s">
+      <c r="D24" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
       <c r="G24" s="17" t="s">
         <v>74</v>
       </c>
@@ -1895,12 +2064,12 @@
       <c r="C25" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="25" t="s">
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="24" t="s">
         <v>81</v>
       </c>
       <c r="H25" s="18">
@@ -1940,11 +2109,11 @@
       <c r="C26" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
       <c r="G26" s="17" t="s">
         <v>87</v>
       </c>
@@ -1985,11 +2154,11 @@
       <c r="C27" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
       <c r="G27" s="17" t="s">
         <v>93</v>
       </c>
@@ -2027,21 +2196,21 @@
       <c r="AA27" s="3"/>
     </row>
     <row r="28" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="40" t="s">
+      <c r="A28" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
-      <c r="M28" s="28"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="25"/>
+      <c r="M28" s="27"/>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
@@ -2067,11 +2236,11 @@
       <c r="C29" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="40" t="s">
         <v>100</v>
       </c>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
       <c r="G29" s="17" t="s">
         <v>101</v>
       </c>
@@ -2112,11 +2281,11 @@
       <c r="C30" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
       <c r="G30" s="17" t="s">
         <v>107</v>
       </c>
@@ -2147,20 +2316,22 @@
       <c r="Z30" s="3"/>
       <c r="AA30" s="3"/>
     </row>
-    <row r="31" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" s="21"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="3"/>
-      <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
+    <row r="31" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="25"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="27"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
@@ -2176,20 +2347,36 @@
       <c r="Z31" s="3"/>
       <c r="AA31" s="3"/>
     </row>
-    <row r="32" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
+    <row r="32" spans="1:27" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D32" s="40" t="s">
+        <v>113</v>
+      </c>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="H32" s="18">
+        <v>46242</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="J32" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="K32" s="18"/>
+      <c r="L32" s="14"/>
+      <c r="M32" s="22"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
@@ -2205,20 +2392,36 @@
       <c r="Z32" s="3"/>
       <c r="AA32" s="3"/>
     </row>
-    <row r="33" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
+    <row r="33" spans="1:27" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D33" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="H33" s="18">
+        <v>46242</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="J33" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="K33" s="18"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="22"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
@@ -2234,20 +2437,36 @@
       <c r="Z33" s="3"/>
       <c r="AA33" s="3"/>
     </row>
-    <row r="34" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
+    <row r="34" spans="1:27" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="D34" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="H34" s="18">
+        <v>46242</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="J34" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="K34" s="18"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="22"/>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
@@ -2263,20 +2482,36 @@
       <c r="Z34" s="3"/>
       <c r="AA34" s="3"/>
     </row>
-    <row r="35" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-      <c r="K35" s="3"/>
-      <c r="L35" s="3"/>
-      <c r="M35" s="3"/>
+    <row r="35" spans="1:27" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="D35" s="40" t="s">
+        <v>131</v>
+      </c>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="H35" s="18">
+        <v>46242</v>
+      </c>
+      <c r="I35" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="J35" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="K35" s="18"/>
+      <c r="L35" s="14"/>
+      <c r="M35" s="22"/>
       <c r="N35" s="3"/>
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
@@ -2293,19 +2528,21 @@
       <c r="AA35" s="3"/>
     </row>
     <row r="36" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
+      <c r="A36" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="25"/>
+      <c r="K36" s="25"/>
+      <c r="L36" s="25"/>
+      <c r="M36" s="27"/>
       <c r="N36" s="3"/>
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
@@ -2321,20 +2558,42 @@
       <c r="Z36" s="3"/>
       <c r="AA36" s="3"/>
     </row>
-    <row r="37" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
-      <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
+    <row r="37" spans="1:27" ht="186.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D37" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="E37" s="25"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="H37" s="18">
+        <v>46242</v>
+      </c>
+      <c r="I37" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="J37" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="K37" s="18">
+        <v>46242</v>
+      </c>
+      <c r="L37" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="M37" s="17" t="s">
+        <v>141</v>
+      </c>
       <c r="N37" s="3"/>
       <c r="O37" s="3"/>
       <c r="P37" s="3"/>
@@ -2350,20 +2609,36 @@
       <c r="Z37" s="3"/>
       <c r="AA37" s="3"/>
     </row>
-    <row r="38" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
+    <row r="38" spans="1:27" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="D38" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="E38" s="25"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="H38" s="18">
+        <v>46242</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="J38" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="K38" s="18"/>
+      <c r="L38" s="14"/>
+      <c r="M38" s="22"/>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
@@ -2380,19 +2655,21 @@
       <c r="AA38" s="3"/>
     </row>
     <row r="39" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
-      <c r="K39" s="3"/>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
+      <c r="A39" s="39" t="s">
+        <v>148</v>
+      </c>
+      <c r="B39" s="25"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="25"/>
+      <c r="J39" s="25"/>
+      <c r="K39" s="25"/>
+      <c r="L39" s="25"/>
+      <c r="M39" s="27"/>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
@@ -2408,20 +2685,36 @@
       <c r="Z39" s="3"/>
       <c r="AA39" s="3"/>
     </row>
-    <row r="40" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
-      <c r="K40" s="3"/>
-      <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
+    <row r="40" spans="1:27" ht="156.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="D40" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="E40" s="25"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="H40" s="18">
+        <v>46242</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="J40" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="K40" s="18"/>
+      <c r="L40" s="14"/>
+      <c r="M40" s="22"/>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
@@ -2734,7 +3027,7 @@
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
+      <c r="G51" s="21"/>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
@@ -2763,7 +3056,7 @@
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
-      <c r="G52" s="21"/>
+      <c r="G52" s="3"/>
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
@@ -30364,47 +30657,28 @@
       <c r="Z1003" s="3"/>
       <c r="AA1003" s="3"/>
     </row>
-    <row r="1004" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A1004" s="3"/>
-      <c r="B1004" s="3"/>
-      <c r="C1004" s="3"/>
-      <c r="D1004" s="3"/>
-      <c r="E1004" s="3"/>
-      <c r="F1004" s="3"/>
-      <c r="G1004" s="3"/>
-      <c r="H1004" s="3"/>
-      <c r="I1004" s="3"/>
-      <c r="J1004" s="3"/>
-      <c r="K1004" s="3"/>
-      <c r="L1004" s="3"/>
-      <c r="M1004" s="3"/>
-      <c r="N1004" s="3"/>
-      <c r="O1004" s="3"/>
-      <c r="P1004" s="3"/>
-      <c r="Q1004" s="3"/>
-      <c r="R1004" s="3"/>
-      <c r="S1004" s="3"/>
-      <c r="T1004" s="3"/>
-      <c r="U1004" s="3"/>
-      <c r="V1004" s="3"/>
-      <c r="W1004" s="3"/>
-      <c r="X1004" s="3"/>
-      <c r="Y1004" s="3"/>
-      <c r="Z1004" s="3"/>
-      <c r="AA1004" s="3"/>
-    </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="47">
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="A31:M31"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="A36:M36"/>
+    <mergeCell ref="A39:M39"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="A28:M28"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="D37:F37"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A23:M23"/>
     <mergeCell ref="N23:Z23"/>
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="A28:M28"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="D30:F30"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="A23:M23"/>
     <mergeCell ref="A18:M18"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="D20:F20"/>
@@ -30452,6 +30726,14 @@
     <hyperlink ref="M27" r:id="rId16" xr:uid="{00000000-0004-0000-0700-00000F000000}"/>
     <hyperlink ref="G29" r:id="rId17" xr:uid="{00000000-0004-0000-0700-000010000000}"/>
     <hyperlink ref="G30" r:id="rId18" xr:uid="{00000000-0004-0000-0700-000011000000}"/>
+    <hyperlink ref="G32" r:id="rId19" xr:uid="{00000000-0004-0000-0700-000012000000}"/>
+    <hyperlink ref="G33" r:id="rId20" xr:uid="{00000000-0004-0000-0700-000013000000}"/>
+    <hyperlink ref="G34" r:id="rId21" xr:uid="{00000000-0004-0000-0700-000014000000}"/>
+    <hyperlink ref="G35" r:id="rId22" xr:uid="{00000000-0004-0000-0700-000015000000}"/>
+    <hyperlink ref="G37" r:id="rId23" xr:uid="{00000000-0004-0000-0700-000016000000}"/>
+    <hyperlink ref="M37" r:id="rId24" xr:uid="{00000000-0004-0000-0700-000017000000}"/>
+    <hyperlink ref="G38" r:id="rId25" xr:uid="{00000000-0004-0000-0700-000018000000}"/>
+    <hyperlink ref="G40" r:id="rId26" xr:uid="{00000000-0004-0000-0700-000019000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor selenium tests and improve test reporting
</commit_message>
<xml_diff>
--- a/TestCases/Doctor_Schedule_Admin_TestCase.xlsx
+++ b/TestCases/Doctor_Schedule_Admin_TestCase.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8696F6DC-1BC0-4181-BEAB-1DE19EB0C63E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D3FECA-98FA-4F37-B4E9-1D14F29FEE7C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="DS_ADMIN" sheetId="8" r:id="rId1"/>
+    <sheet name="DS_ADMIN" sheetId="9" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="ACTION">#REF!</definedName>
@@ -37,16 +37,16 @@
     <t>Module Code：</t>
   </si>
   <si>
-    <t>Test requirement:</t>
+    <t>Pass</t>
   </si>
   <si>
-    <t>Pass</t>
+    <t>Fail</t>
   </si>
   <si>
     <t>Pending</t>
   </si>
   <si>
-    <t>Fail</t>
+    <t>Test requirement:</t>
   </si>
   <si>
     <t>Number of test cases:</t>
@@ -85,10 +85,10 @@
     <t>Retest Evidence</t>
   </si>
   <si>
-    <t>SCHEDULE400 - Doctor Schedule Management</t>
+    <t>SCHEDULE - Doctor Schedule Management</t>
   </si>
   <si>
-    <t>SCHEDULE1 - Manage Doctor Work Schedule</t>
+    <t>Doctor Schedule Management</t>
   </si>
   <si>
     <t>1. Kiểm tra hiển thị form Thêm lịch làm việc</t>
@@ -97,19 +97,19 @@
     <t>TC-DS-ADMIN-001</t>
   </si>
   <si>
-    <t>Kiểm tra form Thêm lịch làm việc hiển thị đầy đủ các trường, danh sách lựa chọn và giá trị mặc định.</t>
+    <t>Kiểm tra form Thêm lịch làm việc hiển thị đầy đủ thông tin cần thiết.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng tài khoản Admin.
-2: Mở trang Quản lý lịch làm việc.
-3: Quan sát các trường và nút trên form Thêm lịch làm việc.
-4: Mở danh sách Bác sĩ và kiểm tra các lựa chọn.
-5: Mở danh sách Ca làm việc và kiểm tra các lựa chọn.
-6: Mở danh sách Trạng thái và kiểm tra các lựa chọn.
-7: Quan sát các giá trị mặc định của form.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Quan sát form Thêm lịch làm việc.
+4: Mở danh sách Bác sĩ.
+5: Mở danh sách Ca làm việc.
+6: Mở danh sách Trạng thái.
+7: Kiểm tra các trường, lựa chọn và giá trị mặc định trên form.</t>
   </si>
   <si>
-    <t>Hiển thị đầy đủ các trường Bác sĩ, Ngày làm việc, Ca làm việc, Trạng thái, Ghi chú và nút Thêm lịch; hiển thị đúng danh sách 4 bác sĩ; Bác sĩ mặc định là -- Chọn bác sĩ --; Ngày làm việc để trống; Ca mặc định là Ca sáng và có đủ 3 ca làm việc; Trạng thái mặc định là Có lịch làm việc và có đủ 2 trạng thái; Ghi chú để trống.</t>
+    <t>Form hiển thị đầy đủ các trường Bác sĩ, Ngày làm việc, Ca làm việc, Trạng thái, Ghi chú và nút Thêm lịch; Bác sĩ mặc định chưa chọn; Ngày làm việc để trống; Ca mặc định là Ca sáng; Trạng thái mặc định là Có lịch làm việc; Ghi chú để trống.</t>
   </si>
   <si>
     <t>TCDsAdmin1_1, TCDsAdmin1_2, TCDsAdmin1_3</t>
@@ -124,21 +124,21 @@
     <t>TC-DS-ADMIN-002</t>
   </si>
   <si>
-    <t>Admin thêm lịch ca sáng với trạng thái Có lịch làm việc và dữ liệu hợp lệ.</t>
+    <t>Kiểm tra Admin thêm lịch làm việc cho bác sĩ với dữ liệu hợp lệ.</t>
   </si>
   <si>
-    <t>1: Chọn bác sĩ Tran Binh.
-2: Nhập ngày 08/08/2026, hiện chưa có lịch
-3: Chọn Ca sáng: 07:00 - 11:30.
-4: Chọn trạng thái Có lịch làm việc.
-5: Nhập ghi chú Ca sáng.
-6: Nhấn nút Thêm lịch.
-7: Chuyển đến tuần chứa ngày vừa chọn nếu cần.
-8: Kiểm tra bảng Lịch làm việc theo tuần.
-9: Kiểm tra Danh sách lịch làm việc.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một bác sĩ.
+4: Chọn một ngày làm việc chưa có lịch tại ca cần tạo.
+5: Chọn Ca sáng.
+6: Chọn trạng thái Có lịch làm việc.
+7: Nhập ghi chú cho lịch.
+8: Nhấn Thêm lịch.
+9: Kiểm tra thông báo và lịch vừa tạo trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Thêm lịch thành công và hiển thị đúng bác sĩ, ngày, ca, trạng thái, ghi chú.</t>
+    <t>Hệ thống thêm lịch thành công và lịch mới hiển thị đúng bác sĩ, ngày, ca, trạng thái và ghi chú đã nhập.</t>
   </si>
   <si>
     <t>TCDsAdmin2</t>
@@ -153,21 +153,20 @@
     <t>TC-DS-ADMIN-003</t>
   </si>
   <si>
-    <t>Kiểm tra Admin có thể thêm lịch với trạng thái Không làm việc.</t>
+    <t>Kiểm tra Admin thêm lịch cho bác sĩ với trạng thái Không làm việc.</t>
   </si>
   <si>
-    <t>1: Chọn bác sĩ Tran Binh.
-2: Nhập ngày 08/08/2026 (bác sĩ chưa có lịch trong ca này).
-3: Chọn Ca tối: 17:30 - 21:00.
-4: Chọn trạng thái Không làm việc.
-5: Nhập ghi chú Không trực.
-6: Nhấn nút Thêm lịch.
-7: Chuyển đến tuần chứa ngày vừa chọn nếu cần.
-8: Kiểm tra bảng Lịch làm việc theo tuần.
-9: Kiểm tra Danh sách lịch làm việc.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một bác sĩ.
+4: Chọn ngày và ca chưa có lịch.
+5: Chọn trạng thái Không làm việc.
+6: Nhập ghi chú phù hợp.
+7: Nhấn Thêm lịch.
+8: Kiểm tra thông báo và lịch vừa tạo trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Thêm lịch thành công với trạng thái Không làm việc và ghi chú Không trực.</t>
+    <t>Hệ thống thêm lịch thành công với trạng thái Không làm việc và lưu đúng thông tin đã nhập.</t>
   </si>
   <si>
     <t>TCDsAdmin3</t>
@@ -179,17 +178,19 @@
     <t>TC-DS-ADMIN-004</t>
   </si>
   <si>
-    <t>Kiểm tra Admin có thể thêm lịch để trống ô ghi chú.</t>
+    <t>Kiểm tra Admin có thể thêm lịch khi để trống Ghi chú.</t>
   </si>
   <si>
-    <t>1: Chọn bác sĩ Tran Binh, ngày 08/08/2026 và Ca tối.
-2: Chọn trạng thái Có lịch làm việc.
-3: Để trống Ghi chú.
-4: Nhấn Thêm lịch.
-5: Kiểm tra lịch vừa tạo.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn bác sĩ, ngày làm việc và ca chưa có lịch.
+4: Chọn trạng thái Có lịch làm việc.
+5: Để trống trường Ghi chú.
+6: Nhấn Thêm lịch.
+7: Kiểm tra lịch vừa tạo trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Lịch vẫn được thêm thành công và cột Ghi chú để trống.</t>
+    <t>Hệ thống vẫn thêm lịch thành công và trường Ghi chú của lịch để trống.</t>
   </si>
   <si>
     <t>TCDsAdmin4</t>
@@ -204,17 +205,19 @@
     <t>TC-DS-ADMIN-005</t>
   </si>
   <si>
-    <t>Kiểm tra hệ thống xử lý khi Admin chưa chọn bác sĩ.</t>
+    <t>Kiểm tra hệ thống xử lý khi Admin không chọn bác sĩ.</t>
   </si>
   <si>
-    <t>1: Giữ trường Bác sĩ ở -- Chọn bác sĩ --.
-2: Chọn ngày làm việc hợp lệ.
-3: Giữ nguyên ca và trạng thái mặc định.
-4: Nhập ghi chú Ca sáng
-5: Nhấn Thêm lịch.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Giữ trường Bác sĩ ở giá trị -- Chọn bác sĩ --.
+4: Chọn ngày làm việc hợp lệ.
+5: Giữ nguyên ca và trạng thái mặc định.
+6: Nhấn Thêm lịch.
+7: Kiểm tra phản hồi tại trường Bác sĩ và Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Hiển thị yêu cầu chọn bác sĩ và không tạo lịch mới.</t>
+    <t>Hệ thống yêu cầu chọn bác sĩ và không tạo lịch mới.</t>
   </si>
   <si>
     <t>TCDsAdmin5</t>
@@ -226,17 +229,19 @@
     <t>TC-DS-ADMIN-006</t>
   </si>
   <si>
-    <t>Kiểm tra hệ thống xử lý khi Admin chưa chọn ngày làm việc.</t>
+    <t>Kiểm tra hệ thống xử lý khi Admin không chọn ngày làm việc.</t>
   </si>
   <si>
-    <t>1: Chọn bác sĩ Tran Binh
-2: Để trống Ngày làm việc
-3: Giữ nguyên ca và trạng thái mặc định.
-4: Nhập ghi chú Ca sáng
-5: Nhấn Thêm lịch.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một bác sĩ.
+4: Để trống trường Ngày làm việc.
+5: Giữ nguyên ca và trạng thái mặc định.
+6: Nhấn Thêm lịch.
+7: Kiểm tra phản hồi tại trường Ngày làm việc và Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Hiển thị yêu cầu chọn ngày và không tạo lịch mới.</t>
+    <t>Hệ thống yêu cầu chọn ngày làm việc và không tạo lịch mới.</t>
   </si>
   <si>
     <t>TCDsAdmin6</t>
@@ -251,17 +256,19 @@
     <t>TC-DS-ADMIN-007</t>
   </si>
   <si>
-    <t>Kiểm tra hệ thống có ngăn tạo lịch làm việc cho ngày đã qua hay không.</t>
+    <t>Kiểm tra hệ thống không cho phép Admin tạo lịch làm việc cho ngày đã qua.</t>
   </si>
   <si>
-    <t>1: Chọn bác sĩ Tran Binh.
-2: Nhập ngày 01/08/2026, hiện chưa có lịch
-3: Giữ nguyên ca và trạng thái mặc định.
-4: Nhập ghi chú Ca sáng.
-5: Nhấn nút Thêm lịch.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một bác sĩ.
+4: Chọn một ngày trước ngày hiện tại.
+5: Chọn ca và trạng thái hợp lệ.
+6: Nhấn Thêm lịch.
+7: Kiểm tra thông báo và Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Không tạo lịch và hiển thị thông báo ngày làm việc không hợp lệ.</t>
+    <t>Hệ thống không tạo lịch cho ngày đã qua và hiển thị thông báo ngày làm việc không hợp lệ.</t>
   </si>
   <si>
     <t>TCDsAdmin7_1, TCDsAdmin7_2</t>
@@ -276,20 +283,21 @@
     <t>TC-DS-ADMIN-008</t>
   </si>
   <si>
-    <t>Kiểm tra không cho phép tạo hai lịch trùng hoàn toàn cho cùng một bác sĩ.</t>
+    <t>Kiểm tra hệ thống không cho phép tạo lịch trùng cho cùng bác sĩ, ngày và ca.</t>
   </si>
   <si>
-    <t>1: Chọn bác sĩ Tran Binh.
-2: Nhập ngày 08/08/2026, hiện chưa có lịch
-3: Chọn Ca tối: 17:30 - 21:00.
-4: Chọn trạng thái Có lịch làm việc.
-5: Nhập ghi chú Ca tối.
-6: Nhấn nút Thêm lịch.
-7: Nhập lại cùng bác sĩ, ngày, ca, trạng thái và ghi chú rồi nhấn Thêm lịch.
-8: Kiểm tra Danh sách lịch làm việc.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một bác sĩ.
+4: Chọn ngày và ca chưa có lịch.
+5: Chọn trạng thái và nhập ghi chú.
+6: Nhấn Thêm lịch.
+7: Nhập lại cùng bác sĩ, cùng ngày và cùng ca.
+8: Nhấn Thêm lịch lần nữa.
+9: Kiểm tra thông báo và các bản ghi trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Không tạo lịch mới và hiển thị thông báo lịch đã tồn tại.</t>
+    <t>Hệ thống không tạo thêm lịch trùng và chỉ tồn tại một lịch cho cùng bác sĩ, ngày và ca.</t>
   </si>
   <si>
     <t>TCDsAdmin8_1, TCDsAdmin8_2</t>
@@ -304,16 +312,19 @@
     <t>TC-DS-ADMIN-009</t>
   </si>
   <si>
-    <t>Kiểm tra một bác sĩ được phép làm nhiều ca khác nhau trong cùng ngày.</t>
+    <t>Kiểm tra một bác sĩ có thể được xếp nhiều ca khác nhau trong cùng ngày.</t>
   </si>
   <si>
-    <t xml:space="preserve">1: Đảm bảo bác sĩ Tran Binh đã có lịch Ca tối ngày 08/08/2026.
-2: Thêm lịch Ca chiều cho Tran Binh cùng ngày.
-3: Kiểm tra bảng tuần và Danh sách lịch làm việc.
-</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Xác định một bác sĩ đã có lịch ở một ca trong ngày.
+4: Chọn cùng bác sĩ và cùng ngày.
+5: Chọn một ca khác với ca đã có.
+6: Nhấn Thêm lịch.
+7: Kiểm tra các lịch của bác sĩ trong Danh sách lịch làm việc và bảng lịch theo tuần.</t>
   </si>
   <si>
-    <t>Ca chiều được thêm thành công và không ảnh hưởng đến lịch Ca tối đã tồn tại.</t>
+    <t>Ca mới được thêm thành công và lịch ở ca trước vẫn được giữ nguyên.</t>
   </si>
   <si>
     <t>TCDsAdmin9_1, TCDsAdmin9_2</t>
@@ -325,15 +336,20 @@
     <t>TC-DS-ADMIN-010</t>
   </si>
   <si>
-    <t>Kiểm tra nhiều bác sĩ được phép làm cùng một ngày và cùng ca.</t>
+    <t>Kiểm tra nhiều bác sĩ có thể được xếp cùng ngày và cùng ca.</t>
   </si>
   <si>
-    <t>1: Thêm lịch Ca sáng cho bác sĩ Tran Binh vào ngày chưa có lịch.
-2: Thêm lịch Ca sáng cho bác sĩ Ly Minh trong cùng ngày.
-3: Kiểm tra bảng tuần và Danh sách lịch làm việc.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn bác sĩ thứ nhất.
+4: Chọn ngày, ca và trạng thái hợp lệ rồi nhấn Thêm lịch.
+5: Chọn bác sĩ thứ hai.
+6: Chọn cùng ngày và cùng ca với bác sĩ thứ nhất.
+7: Chọn trạng thái và nhấn Thêm lịch.
+8: Kiểm tra các lịch trong Danh sách lịch làm việc và bảng lịch theo tuần.</t>
   </si>
   <si>
-    <t>Lịch được thêm và hiển thị đầy đủ cả hai bác sĩ trong cùng ca.</t>
+    <t>Hệ thống thêm lịch thành công cho bác sĩ thứ hai và cả hai bác sĩ đều có lịch độc lập trong cùng ngày, cùng ca.</t>
   </si>
   <si>
     <t>TCDsAdmin10_1, TCDsAdmin10_2</t>
@@ -345,19 +361,21 @@
     <t>TC-DS-ADMIN-011</t>
   </si>
   <si>
-    <t>Kiểm tra hệ thống không cho phép tồn tại hai lịch có trạng thái mâu thuẫn cho cùng bác sĩ, cùng ngày và cùng ca.</t>
+    <t>Kiểm tra không cho phép tạo hai lịch có trạng thái khác nhau cho cùng bác sĩ, ngày và ca.</t>
   </si>
   <si>
-    <t>1: Chọn bác sĩ Tran Binh.
-2: Chọn ngày làm việc chưa có lịch.
-3: Chọn Ca sáng, trạng thái Có lịch làm việc, nhập ghi chú Ca sáng.
-4: Nhấn Thêm lịch và xác nhận lịch được tạo thành công.
-5: Nhập lại cùng bác sĩ, cùng ngày và cùng Ca sáng.
-6: Chọn trạng thái Không làm việc, nhập ghi chú Nghỉ phép.
-7: Nhấn Thêm lịch và kiểm tra Danh sách lịch làm việc.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một bác sĩ.
+4: Chọn ngày và ca chưa có lịch.
+5: Chọn trạng thái Có lịch làm việc và nhấn Thêm lịch.
+6: Chọn lại cùng bác sĩ, cùng ngày và cùng ca.
+7: Chọn trạng thái Không làm việc.
+8: Nhấn Thêm lịch.
+9: Kiểm tra thông báo và các bản ghi trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Hệ thống không tạo thêm bản ghi mới. Cùng một bác sĩ, ngày và ca chỉ được tồn tại một trạng thái lịch; nếu muốn thay đổi trạng thái thì phải cập nhật lịch hiện có.</t>
+    <t>Hệ thống không tạo thêm lịch có trạng thái khác cho cùng bác sĩ, ngày và ca.</t>
   </si>
   <si>
     <t>TCDsAdmin11</t>
@@ -375,16 +393,17 @@
     <t>TC-DS-ADMIN-012</t>
   </si>
   <si>
-    <t>Kiểm tra hệ thống không tạo nhiều bản ghi khi nhấn nút Thêm lịch liên tục.</t>
+    <t>Kiểm tra hệ thống không tạo nhiều lịch khi Admin nhấn nút Thêm lịch liên tục.</t>
   </si>
   <si>
-    <t>1: Nhập dữ liệu hợp lệ cho một lịch chưa tồn tại.
-2: Nhấn nhanh nút Thêm lịch nhiều lần.
-3: Chờ hệ thống xử lý.
-4: Kiểm tra bảng tuần và danh sách lịch.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn bác sĩ, ngày làm việc, ca, trạng thái và nhập ghi chú hợp lệ cho một lịch chưa tồn tại.
+4: Nhấn nút Thêm lịch nhiều lần liên tục.
+5: Kiểm tra số bản ghi tương ứng trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Chỉ tạo một lịch làm việc.</t>
+    <t>Hệ thống chỉ tạo một lịch làm việc từ thao tác trên.</t>
   </si>
   <si>
     <t>TCDsAdmin12_1, TCDsAdmin12_2, TCDsAdmin12_3</t>
@@ -399,13 +418,14 @@
     <t>Kiểm tra form trở về trạng thái mặc định sau khi thêm lịch thành công.</t>
   </si>
   <si>
-    <t>1: Nhập dữ liệu hợp lệ cho một lịch chưa tồn tại.
-2: Nhấn Thêm lịch.
-3: Chờ thông báo thành công.
-4: Quan sát lại các trường trên form.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn bác sĩ, ngày làm việc, ca, trạng thái và nhập ghi chú hợp lệ cho một lịch chưa tồn tại.
+4: Nhấn Thêm lịch.
+5: Kiểm tra lại các trường trên form Thêm lịch làm việc sau khi thao tác hoàn tất.</t>
   </si>
   <si>
-    <t>Sau khi thêm lịch thành công, form trở về trạng thái mặc định: Bác sĩ chưa chọn; Ngày làm việc trống; Ca làm việc = Ca sáng 07:00–11:30; Trạng thái = Có lịch làm việc; Ghi chú trống; nút Thêm lịch tiếp tục hiển thị.</t>
+    <t>Form trở về trạng thái mặc định: chưa chọn bác sĩ, ngày làm việc trống, Ca sáng, trạng thái Có lịch làm việc và Ghi chú trống.</t>
   </si>
   <si>
     <t>TCDsAdmin13_1, TCDsAdmin13_2</t>
@@ -420,17 +440,17 @@
     <t>TC-DS-ADMIN-014</t>
   </si>
   <si>
-    <t>Kiểm tra Admin có thể lọc lịch làm việc theo một bác sĩ cụ thể.</t>
+    <t>Kiểm tra Admin lọc lịch làm việc theo bác sĩ.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng tài khoản Admin.
-2: Mở trang Quản lý lịch làm việc.
-3: Tại mục Lọc lịch làm việc, chọn bác sĩ Tran Binh.
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Tại mục Lọc lịch làm việc, chọn một bác sĩ có lịch trong tuần đang xem.
 4: Quan sát bảng Lịch làm việc theo tuần.
-5: Kiểm tra các lịch đang hiển thị trong tuần hiện tại.</t>
+5: Kiểm tra bác sĩ của các lịch đang hiển thị.</t>
   </si>
   <si>
-    <t>Bảng Lịch làm việc theo tuần chỉ hiển thị lịch của bác sĩ Tran Binh; lịch của các bác sĩ khác không được hiển thị.</t>
+    <t>Bảng lịch theo tuần chỉ hiển thị lịch của bác sĩ được chọn.</t>
   </si>
   <si>
     <t>TCDsAdmin14</t>
@@ -442,16 +462,18 @@
     <t>TC-DS-ADMIN-015</t>
   </si>
   <si>
-    <t>Kiểm tra hiển thị lại lịch của tất cả bác sĩ sau khi bỏ điều kiện lọc.</t>
+    <t>Kiểm tra Admin hiển thị lại lịch của tất cả bác sĩ sau khi bỏ điều kiện lọc.</t>
   </si>
   <si>
-    <t>1: Tại mục Lọc lịch làm việc, chọn bác sĩ Tran Binh.
-2: Xác nhận bảng tuần chỉ hiển thị lịch của Tran Binh.
-3: Chọn lại Tất cả bác sĩ.
-4: Quan sát bảng Lịch làm việc theo tuần.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một bác sĩ tại mục Lọc lịch làm việc.
+4: Kiểm tra dữ liệu đang được lọc theo bác sĩ đã chọn.
+5: Chọn lại Tất cả bác sĩ.
+6: Kiểm tra bảng Lịch làm việc theo tuần.</t>
   </si>
   <si>
-    <t>Hệ thống bỏ điều kiện lọc và hiển thị lại lịch làm việc của tất cả bác sĩ trong tuần đang xem.</t>
+    <t>Hệ thống bỏ điều kiện lọc và hiển thị lại lịch của tất cả bác sĩ trong tuần đang xem.</t>
   </si>
   <si>
     <t>TCDsAdmin15_1, TCDsAdmin15_2</t>
@@ -463,17 +485,17 @@
     <t>TC-DS-ADMIN-016</t>
   </si>
   <si>
-    <t>Kiểm tra Admin có thể chuyển sang tuần trước để xem lịch làm việc.</t>
+    <t>Kiểm tra Admin chuyển sang tuần trước để xem lịch làm việc.</t>
   </si>
   <si>
-    <t>1: Mở trang Quản lý lịch làm việc.
-2: Ghi nhận khoảng thời gian của tuần đang hiển thị.
-3: Nhấn nút Tuần trước.
-4: Quan sát khoảng thời gian tại mục Tuần làm việc.
-5: Quan sát ngày và dữ liệu trong bảng Lịch làm việc theo tuần.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Ghi nhận khoảng ngày của tuần đang hiển thị.
+4: Nhấn Tuần trước.
+5: Kiểm tra khoảng ngày và dữ liệu trong bảng Lịch làm việc theo tuần.</t>
   </si>
   <si>
-    <t>Hệ thống chuyển về tuần liền trước; khoảng ngày và các cột ngày trong bảng tuần được cập nhật đúng theo tuần mới; dữ liệu lịch hiển thị tương ứng với tuần được chọn.</t>
+    <t>Hệ thống chuyển về tuần liền trước, cập nhật đúng khoảng ngày và hiển thị dữ liệu lịch của tuần đó.</t>
   </si>
   <si>
     <t>TCDsAdmin16_1, TCDsAdmin16_2</t>
@@ -485,17 +507,17 @@
     <t>TC-DS-ADMIN-017</t>
   </si>
   <si>
-    <t>Kiểm tra Admin có thể chuyển sang tuần sau để xem lịch làm việc.</t>
+    <t>Kiểm tra Admin chuyển sang tuần sau để xem lịch làm việc.</t>
   </si>
   <si>
-    <t>1: Mở trang Quản lý lịch làm việc.
-2: Ghi nhận khoảng thời gian của tuần đang hiển thị.
-3: Nhấn nút Tuần sau.
-4: Quan sát khoảng thời gian tại mục Tuần làm việc.
-5: Quan sát ngày và dữ liệu trong bảng Lịch làm việc theo tuần.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Ghi nhận khoảng ngày của tuần đang hiển thị.
+4: Nhấn Tuần sau.
+5: Kiểm tra khoảng ngày và dữ liệu trong bảng Lịch làm việc theo tuần.</t>
   </si>
   <si>
-    <t>Hệ thống chuyển sang tuần liền sau; khoảng ngày và các cột ngày trong bảng tuần được cập nhật đúng theo tuần mới; dữ liệu lịch hiển thị tương ứng với tuần được chọn.</t>
+    <t>Hệ thống chuyển sang tuần liền sau, cập nhật đúng khoảng ngày và hiển thị dữ liệu lịch của tuần đó.</t>
   </si>
   <si>
     <t>TCDsAdmin17_1, TCDsAdmin17_2</t>
@@ -510,21 +532,20 @@
     <t>TC-DS-ADMIN-018</t>
   </si>
   <si>
-    <t>Kiểm tra Admin cập nhật lịch làm việc của bác sĩ thành công.</t>
+    <t>Kiểm tra Admin cập nhật lịch làm việc đã tồn tại của bác sĩ.</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng tài khoản Admin.
-2: Mở trang Quản lý lịch làm việc.
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
 3: Tại Danh sách lịch làm việc, chọn một lịch đã tồn tại và nhấn Sửa.
-4: Kiểm tra thông tin lịch được hiển thị trên form Cập nhật lịch làm việc.
-5: Thay đổi Trạng thái từ Có lịch làm việc thành Không làm việc.
-6: Thay đổi Ghi chú thành Nghỉ.
+4: Kiểm tra thông tin lịch được đưa lên form Cập nhật lịch làm việc.
+5: Thay đổi trạng thái của lịch.
+6: Thay đổi Ghi chú.
 7: Nhấn Cập nhật.
-8: Kiểm tra thông báo của hệ thống.
-9: Kiểm tra lại lịch trong Danh sách lịch làm việc và bảng Lịch làm việc theo tuần.</t>
+8: Kiểm tra thông báo và thông tin lịch sau khi cập nhật trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Hệ thống cập nhật lịch thành công; trạng thái và ghi chú được thay đổi đúng, không tạo thêm bản ghi mới và thông tin được hiển thị đúng trong danh sách và bảng tuần.</t>
+    <t>Hệ thống cập nhật lịch thành công, lưu đúng thông tin mới và không tạo thêm bản ghi lịch khác.</t>
   </si>
   <si>
     <t>TCDsAdmin18_1, TCDsAdmin18_2</t>
@@ -539,18 +560,19 @@
     <t>TC-DS-ADMIN-019</t>
   </si>
   <si>
-    <t>Kiểm tra chức năng Hủy sửa không làm thay đổi dữ liệu lịch.</t>
+    <t>Kiểm tra Hủy sửa không làm thay đổi thông tin lịch làm việc.</t>
   </si>
   <si>
-    <t>1: Chọn một lịch hiện có trong Danh sách lịch làm việc và ghi nhận thông tin ban đầu.
-2: Nhấn Sửa.
-3: Thay đổi một số giá trị trên form nhưng chưa nhấn Cập nhật.
-4: Nhấn Hủy sửa.
-5: Quan sát lại form.
-6: Kiểm tra lịch tương ứng trong Danh sách lịch làm việc.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Chọn một lịch trong Danh sách lịch làm việc và ghi nhận thông tin ban đầu.
+4: Nhấn Sửa.
+5: Thay đổi một số thông tin trên form nhưng chưa nhấn Cập nhật.
+6: Nhấn Hủy sửa.
+7: Kiểm tra form và thông tin của lịch trong Danh sách lịch làm việc.</t>
   </si>
   <si>
-    <t>Hệ thống thoát chế độ cập nhật và đưa form về trạng thái thêm lịch mặc định; các thay đổi chưa được lưu không làm thay đổi dữ liệu của lịch trong Danh sách lịch làm việc.</t>
+    <t>Form thoát khỏi chế độ cập nhật, trở về trạng thái thêm lịch và dữ liệu của lịch ban đầu không bị thay đổi.</t>
   </si>
   <si>
     <t>TCDsAdmin19_1, TCDsAdmin19_2, TCDsAdmin19_3</t>
@@ -565,19 +587,19 @@
     <t>TC-DS-ADMIN-020</t>
   </si>
   <si>
-    <t>Kiểm tra Admin có thể xóa một lịch làm việc đã tồn tại.</t>
+    <t>Kiểm tra Admin xóa lịch làm việc đã tồn tại của bác sĩ.</t>
   </si>
   <si>
-    <t>1: Tạo hoặc xác định một lịch dùng riêng cho kiểm thử xóa.
-2: Kiểm tra lịch đang tồn tại trong Danh sách lịch làm việc.
-3: Nhấn nút Xóa tại lịch đó.
-4: Xác nhận thao tác xóa nếu hệ thống yêu cầu xác nhận.
-5: Chờ hệ thống xử lý.
-6: Kiểm tra lại Danh sách lịch làm việc.
-7: Kiểm tra bảng Lịch làm việc theo tuần.</t>
+    <t>1: Đăng nhập với vai trò Admin.
+2: Mở trang Quản lý lịch làm việc bác sĩ.
+3: Xác định một lịch dùng cho kiểm thử xóa trong Danh sách lịch làm việc.
+4: Nhấn Xóa tại lịch đó.
+5: Xác nhận thao tác xóa trên hộp thoại.
+6: Kiểm tra thông báo của hệ thống.
+7: Kiểm tra lại Danh sách lịch làm việc và bảng lịch theo tuần.</t>
   </si>
   <si>
-    <t>Hệ thống xóa lịch thành công; lịch đã xóa không còn xuất hiện trong Danh sách lịch làm việc và không còn hiển thị trong bảng Lịch làm việc theo tuần.</t>
+    <t>Hệ thống xóa lịch thành công; lịch đã xóa không còn xuất hiện trong Danh sách lịch làm việc và bảng lịch theo tuần.</t>
   </si>
   <si>
     <t>TCDsAdmin20_1, TCDsAdmin20_2, TCDsAdmin20_3</t>
@@ -606,10 +628,6 @@
       <name val="Tahoma"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="MS PGothic"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -619,6 +637,10 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="MS PGothic"/>
     </font>
     <font>
       <b/>
@@ -825,10 +847,10 @@
   </cellStyleXfs>
   <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -844,10 +866,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -863,15 +885,15 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -879,34 +901,34 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1125,7 +1147,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -1134,7 +1156,7 @@
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
     <col min="2" max="2" width="22.109375" customWidth="1"/>
-    <col min="3" max="3" width="43.44140625" customWidth="1"/>
+    <col min="3" max="3" width="46.77734375" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="22.6640625" customWidth="1"/>
     <col min="8" max="8" width="20.109375" customWidth="1"/>
@@ -1148,9 +1170,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1177,9 +1199,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1208,11 +1230,11 @@
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="27"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="30"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1241,11 +1263,11 @@
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="27"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="30"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1272,13 +1294,13 @@
     </row>
     <row r="5" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="27"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="30"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1305,7 +1327,7 @@
     </row>
     <row r="6" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="6">
         <v>13</v>
@@ -1342,7 +1364,7 @@
     </row>
     <row r="7" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7" s="6">
         <v>7</v>
@@ -1407,21 +1429,21 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="34" t="s">
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="32" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="37" t="s">
@@ -1458,19 +1480,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
+      <c r="A10" s="33"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="33"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1489,17 +1511,17 @@
     <row r="11" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="38"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
+      <c r="M11" s="29"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1519,18 +1541,18 @@
       <c r="A12" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="27"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="29"/>
+      <c r="K12" s="29"/>
+      <c r="L12" s="29"/>
+      <c r="M12" s="30"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1546,7 +1568,7 @@
       <c r="Z12" s="3"/>
       <c r="AA12" s="3"/>
     </row>
-    <row r="13" spans="1:27" ht="138.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" ht="123" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>23</v>
       </c>
@@ -1559,8 +1581,8 @@
       <c r="D13" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
       <c r="G13" s="17" t="s">
         <v>27</v>
       </c>
@@ -1568,7 +1590,7 @@
         <v>46240</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>28</v>
@@ -1595,18 +1617,18 @@
       <c r="A14" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="25"/>
-      <c r="M14" s="27"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="29"/>
+      <c r="L14" s="29"/>
+      <c r="M14" s="30"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1622,7 +1644,7 @@
       <c r="Z14" s="3"/>
       <c r="AA14" s="3"/>
     </row>
-    <row r="15" spans="1:27" ht="130.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>30</v>
       </c>
@@ -1635,8 +1657,8 @@
       <c r="D15" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
       <c r="G15" s="17" t="s">
         <v>34</v>
       </c>
@@ -1644,7 +1666,7 @@
         <v>46240</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J15" s="16" t="s">
         <v>35</v>
@@ -1653,7 +1675,7 @@
         <v>46240</v>
       </c>
       <c r="L15" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M15" s="17" t="s">
         <v>36</v>
@@ -1673,7 +1695,7 @@
       <c r="Z15" s="3"/>
       <c r="AA15" s="3"/>
     </row>
-    <row r="16" spans="1:27" ht="183.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>37</v>
       </c>
@@ -1686,8 +1708,8 @@
       <c r="D16" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
       <c r="G16" s="17" t="s">
         <v>41</v>
       </c>
@@ -1695,7 +1717,7 @@
         <v>46240</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>35</v>
@@ -1704,7 +1726,7 @@
         <v>46240</v>
       </c>
       <c r="L16" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M16" s="17" t="s">
         <v>42</v>
@@ -1724,7 +1746,7 @@
       <c r="Z16" s="3"/>
       <c r="AA16" s="3"/>
     </row>
-    <row r="17" spans="1:27" ht="183.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>43</v>
       </c>
@@ -1737,8 +1759,8 @@
       <c r="D17" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
       <c r="G17" s="17" t="s">
         <v>47</v>
       </c>
@@ -1746,7 +1768,7 @@
         <v>46240</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J17" s="16" t="s">
         <v>35</v>
@@ -1755,7 +1777,7 @@
         <v>46240</v>
       </c>
       <c r="L17" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M17" s="17" t="s">
         <v>48</v>
@@ -1779,18 +1801,18 @@
       <c r="A18" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="25"/>
-      <c r="M18" s="27"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="29"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="29"/>
+      <c r="M18" s="30"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -1819,8 +1841,8 @@
       <c r="D19" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
       <c r="G19" s="17" t="s">
         <v>54</v>
       </c>
@@ -1828,7 +1850,7 @@
         <v>46240</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J19" s="16" t="s">
         <v>55</v>
@@ -1864,8 +1886,8 @@
       <c r="D20" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
       <c r="G20" s="17" t="s">
         <v>60</v>
       </c>
@@ -1873,7 +1895,7 @@
         <v>46240</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>61</v>
@@ -1900,31 +1922,31 @@
       <c r="A21" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="25"/>
-      <c r="M21" s="27"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
+      <c r="K21" s="29"/>
+      <c r="L21" s="29"/>
+      <c r="M21" s="30"/>
       <c r="N21" s="41"/>
-      <c r="O21" s="31"/>
-      <c r="P21" s="31"/>
-      <c r="Q21" s="31"/>
-      <c r="R21" s="31"/>
-      <c r="S21" s="31"/>
-      <c r="T21" s="31"/>
-      <c r="U21" s="31"/>
-      <c r="V21" s="31"/>
-      <c r="W21" s="31"/>
-      <c r="X21" s="31"/>
-      <c r="Y21" s="31"/>
-      <c r="Z21" s="31"/>
+      <c r="O21" s="25"/>
+      <c r="P21" s="25"/>
+      <c r="Q21" s="25"/>
+      <c r="R21" s="25"/>
+      <c r="S21" s="25"/>
+      <c r="T21" s="25"/>
+      <c r="U21" s="25"/>
+      <c r="V21" s="25"/>
+      <c r="W21" s="25"/>
+      <c r="X21" s="25"/>
+      <c r="Y21" s="25"/>
+      <c r="Z21" s="25"/>
       <c r="AA21" s="3"/>
     </row>
     <row r="22" spans="1:27" ht="128.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1940,8 +1962,8 @@
       <c r="D22" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
       <c r="G22" s="23" t="s">
         <v>67</v>
       </c>
@@ -1949,7 +1971,7 @@
         <v>46240</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>68</v>
@@ -1976,34 +1998,34 @@
       <c r="A23" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
-      <c r="M23" s="27"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="30"/>
       <c r="N23" s="42"/>
-      <c r="O23" s="31"/>
-      <c r="P23" s="31"/>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="31"/>
-      <c r="S23" s="31"/>
-      <c r="T23" s="31"/>
-      <c r="U23" s="31"/>
-      <c r="V23" s="31"/>
-      <c r="W23" s="31"/>
-      <c r="X23" s="31"/>
-      <c r="Y23" s="31"/>
-      <c r="Z23" s="31"/>
+      <c r="O23" s="25"/>
+      <c r="P23" s="25"/>
+      <c r="Q23" s="25"/>
+      <c r="R23" s="25"/>
+      <c r="S23" s="25"/>
+      <c r="T23" s="25"/>
+      <c r="U23" s="25"/>
+      <c r="V23" s="25"/>
+      <c r="W23" s="25"/>
+      <c r="X23" s="25"/>
+      <c r="Y23" s="25"/>
+      <c r="Z23" s="25"/>
       <c r="AA23" s="3"/>
     </row>
-    <row r="24" spans="1:27" ht="126" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" ht="139.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>70</v>
       </c>
@@ -2016,8 +2038,8 @@
       <c r="D24" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
       <c r="G24" s="17" t="s">
         <v>74</v>
       </c>
@@ -2025,7 +2047,7 @@
         <v>46240</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J24" s="16" t="s">
         <v>75</v>
@@ -2034,7 +2056,7 @@
         <v>46241</v>
       </c>
       <c r="L24" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M24" s="17" t="s">
         <v>76</v>
@@ -2067,8 +2089,8 @@
       <c r="D25" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
       <c r="G25" s="24" t="s">
         <v>81</v>
       </c>
@@ -2076,14 +2098,14 @@
         <v>46240</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J25" s="16" t="s">
         <v>82</v>
       </c>
       <c r="K25" s="18"/>
       <c r="L25" s="14"/>
-      <c r="M25" s="22"/>
+      <c r="M25" s="21"/>
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
@@ -2112,8 +2134,8 @@
       <c r="D26" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
       <c r="G26" s="17" t="s">
         <v>87</v>
       </c>
@@ -2121,14 +2143,14 @@
         <v>46240</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J26" s="16" t="s">
         <v>88</v>
       </c>
       <c r="K26" s="18"/>
       <c r="L26" s="14"/>
-      <c r="M26" s="22"/>
+      <c r="M26" s="21"/>
       <c r="N26" s="3"/>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
@@ -2157,8 +2179,8 @@
       <c r="D27" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
       <c r="G27" s="17" t="s">
         <v>93</v>
       </c>
@@ -2166,7 +2188,7 @@
         <v>46240</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>94</v>
@@ -2175,7 +2197,7 @@
         <v>46241</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M27" s="17" t="s">
         <v>95</v>
@@ -2199,18 +2221,18 @@
       <c r="A28" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="25"/>
-      <c r="I28" s="25"/>
-      <c r="J28" s="25"/>
-      <c r="K28" s="25"/>
-      <c r="L28" s="25"/>
-      <c r="M28" s="27"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
+      <c r="K28" s="29"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="30"/>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
@@ -2239,8 +2261,8 @@
       <c r="D29" s="40" t="s">
         <v>100</v>
       </c>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
       <c r="G29" s="17" t="s">
         <v>101</v>
       </c>
@@ -2248,14 +2270,14 @@
         <v>46240</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J29" s="16" t="s">
         <v>102</v>
       </c>
       <c r="K29" s="18"/>
       <c r="L29" s="14"/>
-      <c r="M29" s="22"/>
+      <c r="M29" s="21"/>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
@@ -2284,8 +2306,8 @@
       <c r="D30" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
       <c r="G30" s="17" t="s">
         <v>107</v>
       </c>
@@ -2293,14 +2315,14 @@
         <v>46240</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J30" s="16" t="s">
         <v>108</v>
       </c>
       <c r="K30" s="18"/>
       <c r="L30" s="14"/>
-      <c r="M30" s="22"/>
+      <c r="M30" s="21"/>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
@@ -2320,18 +2342,18 @@
       <c r="A31" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="25"/>
-      <c r="I31" s="25"/>
-      <c r="J31" s="25"/>
-      <c r="K31" s="25"/>
-      <c r="L31" s="25"/>
-      <c r="M31" s="27"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="29"/>
+      <c r="L31" s="29"/>
+      <c r="M31" s="30"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
@@ -2360,8 +2382,8 @@
       <c r="D32" s="40" t="s">
         <v>113</v>
       </c>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
       <c r="G32" s="17" t="s">
         <v>114</v>
       </c>
@@ -2369,14 +2391,14 @@
         <v>46242</v>
       </c>
       <c r="I32" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J32" s="16" t="s">
         <v>115</v>
       </c>
       <c r="K32" s="18"/>
       <c r="L32" s="14"/>
-      <c r="M32" s="22"/>
+      <c r="M32" s="21"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
@@ -2405,8 +2427,8 @@
       <c r="D33" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
       <c r="G33" s="17" t="s">
         <v>120</v>
       </c>
@@ -2414,14 +2436,14 @@
         <v>46242</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J33" s="16" t="s">
         <v>121</v>
       </c>
       <c r="K33" s="18"/>
       <c r="L33" s="14"/>
-      <c r="M33" s="22"/>
+      <c r="M33" s="21"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
@@ -2450,8 +2472,8 @@
       <c r="D34" s="40" t="s">
         <v>125</v>
       </c>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
       <c r="G34" s="17" t="s">
         <v>126</v>
       </c>
@@ -2459,14 +2481,14 @@
         <v>46242</v>
       </c>
       <c r="I34" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J34" s="16" t="s">
         <v>127</v>
       </c>
       <c r="K34" s="18"/>
       <c r="L34" s="14"/>
-      <c r="M34" s="22"/>
+      <c r="M34" s="21"/>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
@@ -2495,8 +2517,8 @@
       <c r="D35" s="40" t="s">
         <v>131</v>
       </c>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
       <c r="G35" s="17" t="s">
         <v>132</v>
       </c>
@@ -2504,14 +2526,14 @@
         <v>46242</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J35" s="16" t="s">
         <v>133</v>
       </c>
       <c r="K35" s="18"/>
       <c r="L35" s="14"/>
-      <c r="M35" s="22"/>
+      <c r="M35" s="21"/>
       <c r="N35" s="3"/>
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
@@ -2531,18 +2553,18 @@
       <c r="A36" s="39" t="s">
         <v>134</v>
       </c>
-      <c r="B36" s="25"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="25"/>
-      <c r="J36" s="25"/>
-      <c r="K36" s="25"/>
-      <c r="L36" s="25"/>
-      <c r="M36" s="27"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+      <c r="J36" s="29"/>
+      <c r="K36" s="29"/>
+      <c r="L36" s="29"/>
+      <c r="M36" s="30"/>
       <c r="N36" s="3"/>
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
@@ -2571,8 +2593,8 @@
       <c r="D37" s="40" t="s">
         <v>138</v>
       </c>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
       <c r="G37" s="17" t="s">
         <v>139</v>
       </c>
@@ -2580,7 +2602,7 @@
         <v>46242</v>
       </c>
       <c r="I37" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J37" s="16" t="s">
         <v>140</v>
@@ -2589,7 +2611,7 @@
         <v>46242</v>
       </c>
       <c r="L37" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M37" s="17" t="s">
         <v>141</v>
@@ -2622,8 +2644,8 @@
       <c r="D38" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="E38" s="25"/>
-      <c r="F38" s="25"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
       <c r="G38" s="17" t="s">
         <v>146</v>
       </c>
@@ -2631,14 +2653,14 @@
         <v>46242</v>
       </c>
       <c r="I38" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J38" s="16" t="s">
         <v>147</v>
       </c>
       <c r="K38" s="18"/>
       <c r="L38" s="14"/>
-      <c r="M38" s="22"/>
+      <c r="M38" s="21"/>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
@@ -2658,18 +2680,18 @@
       <c r="A39" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="B39" s="25"/>
-      <c r="C39" s="25"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="25"/>
-      <c r="J39" s="25"/>
-      <c r="K39" s="25"/>
-      <c r="L39" s="25"/>
-      <c r="M39" s="27"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="29"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="29"/>
+      <c r="H39" s="29"/>
+      <c r="I39" s="29"/>
+      <c r="J39" s="29"/>
+      <c r="K39" s="29"/>
+      <c r="L39" s="29"/>
+      <c r="M39" s="30"/>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
@@ -2698,8 +2720,8 @@
       <c r="D40" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
       <c r="G40" s="17" t="s">
         <v>153</v>
       </c>
@@ -2707,14 +2729,14 @@
         <v>46242</v>
       </c>
       <c r="I40" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J40" s="16" t="s">
         <v>154</v>
       </c>
       <c r="K40" s="18"/>
       <c r="L40" s="14"/>
-      <c r="M40" s="22"/>
+      <c r="M40" s="21"/>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
@@ -3027,7 +3049,7 @@
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
-      <c r="G51" s="21"/>
+      <c r="G51" s="22"/>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
       <c r="J51" s="3"/>
@@ -30708,32 +30730,32 @@
     <mergeCell ref="C9:C10"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
-    <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
-    <hyperlink ref="M15" r:id="rId3" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
-    <hyperlink ref="G16" r:id="rId4" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
-    <hyperlink ref="M16" r:id="rId5" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
-    <hyperlink ref="G17" r:id="rId6" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
-    <hyperlink ref="M17" r:id="rId7" xr:uid="{00000000-0004-0000-0700-000006000000}"/>
-    <hyperlink ref="G19" r:id="rId8" xr:uid="{00000000-0004-0000-0700-000007000000}"/>
-    <hyperlink ref="G20" r:id="rId9" xr:uid="{00000000-0004-0000-0700-000008000000}"/>
-    <hyperlink ref="G22" r:id="rId10" xr:uid="{00000000-0004-0000-0700-000009000000}"/>
-    <hyperlink ref="G24" r:id="rId11" xr:uid="{00000000-0004-0000-0700-00000A000000}"/>
-    <hyperlink ref="M24" r:id="rId12" xr:uid="{00000000-0004-0000-0700-00000B000000}"/>
-    <hyperlink ref="G25" r:id="rId13" xr:uid="{00000000-0004-0000-0700-00000C000000}"/>
-    <hyperlink ref="G26" r:id="rId14" xr:uid="{00000000-0004-0000-0700-00000D000000}"/>
-    <hyperlink ref="G27" r:id="rId15" xr:uid="{00000000-0004-0000-0700-00000E000000}"/>
-    <hyperlink ref="M27" r:id="rId16" xr:uid="{00000000-0004-0000-0700-00000F000000}"/>
-    <hyperlink ref="G29" r:id="rId17" xr:uid="{00000000-0004-0000-0700-000010000000}"/>
-    <hyperlink ref="G30" r:id="rId18" xr:uid="{00000000-0004-0000-0700-000011000000}"/>
-    <hyperlink ref="G32" r:id="rId19" xr:uid="{00000000-0004-0000-0700-000012000000}"/>
-    <hyperlink ref="G33" r:id="rId20" xr:uid="{00000000-0004-0000-0700-000013000000}"/>
-    <hyperlink ref="G34" r:id="rId21" xr:uid="{00000000-0004-0000-0700-000014000000}"/>
-    <hyperlink ref="G35" r:id="rId22" xr:uid="{00000000-0004-0000-0700-000015000000}"/>
-    <hyperlink ref="G37" r:id="rId23" xr:uid="{00000000-0004-0000-0700-000016000000}"/>
-    <hyperlink ref="M37" r:id="rId24" xr:uid="{00000000-0004-0000-0700-000017000000}"/>
-    <hyperlink ref="G38" r:id="rId25" xr:uid="{00000000-0004-0000-0700-000018000000}"/>
-    <hyperlink ref="G40" r:id="rId26" xr:uid="{00000000-0004-0000-0700-000019000000}"/>
+    <hyperlink ref="G13" r:id="rId1" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
+    <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
+    <hyperlink ref="M15" r:id="rId3" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
+    <hyperlink ref="G16" r:id="rId4" xr:uid="{00000000-0004-0000-0800-000003000000}"/>
+    <hyperlink ref="M16" r:id="rId5" xr:uid="{00000000-0004-0000-0800-000004000000}"/>
+    <hyperlink ref="G17" r:id="rId6" xr:uid="{00000000-0004-0000-0800-000005000000}"/>
+    <hyperlink ref="M17" r:id="rId7" xr:uid="{00000000-0004-0000-0800-000006000000}"/>
+    <hyperlink ref="G19" r:id="rId8" xr:uid="{00000000-0004-0000-0800-000007000000}"/>
+    <hyperlink ref="G20" r:id="rId9" xr:uid="{00000000-0004-0000-0800-000008000000}"/>
+    <hyperlink ref="G22" r:id="rId10" xr:uid="{00000000-0004-0000-0800-000009000000}"/>
+    <hyperlink ref="G24" r:id="rId11" xr:uid="{00000000-0004-0000-0800-00000A000000}"/>
+    <hyperlink ref="M24" r:id="rId12" xr:uid="{00000000-0004-0000-0800-00000B000000}"/>
+    <hyperlink ref="G25" r:id="rId13" xr:uid="{00000000-0004-0000-0800-00000C000000}"/>
+    <hyperlink ref="G26" r:id="rId14" xr:uid="{00000000-0004-0000-0800-00000D000000}"/>
+    <hyperlink ref="G27" r:id="rId15" xr:uid="{00000000-0004-0000-0800-00000E000000}"/>
+    <hyperlink ref="M27" r:id="rId16" xr:uid="{00000000-0004-0000-0800-00000F000000}"/>
+    <hyperlink ref="G29" r:id="rId17" xr:uid="{00000000-0004-0000-0800-000010000000}"/>
+    <hyperlink ref="G30" r:id="rId18" xr:uid="{00000000-0004-0000-0800-000011000000}"/>
+    <hyperlink ref="G32" r:id="rId19" xr:uid="{00000000-0004-0000-0800-000012000000}"/>
+    <hyperlink ref="G33" r:id="rId20" xr:uid="{00000000-0004-0000-0800-000013000000}"/>
+    <hyperlink ref="G34" r:id="rId21" xr:uid="{00000000-0004-0000-0800-000014000000}"/>
+    <hyperlink ref="G35" r:id="rId22" xr:uid="{00000000-0004-0000-0800-000015000000}"/>
+    <hyperlink ref="G37" r:id="rId23" xr:uid="{00000000-0004-0000-0800-000016000000}"/>
+    <hyperlink ref="M37" r:id="rId24" xr:uid="{00000000-0004-0000-0800-000017000000}"/>
+    <hyperlink ref="G38" r:id="rId25" xr:uid="{00000000-0004-0000-0800-000018000000}"/>
+    <hyperlink ref="G40" r:id="rId26" xr:uid="{00000000-0004-0000-0800-000019000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>